<commit_message>
Simplify report and workbook formatting
Remove all color, fills, the running header, the cover rule and note,
and the restated question text. Headings are now just the question
numbers. Numbers and wording of the answers are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ShG3KqQSYtUQ4UFSULXCgJ
</commit_message>
<xml_diff>
--- a/Walmart_Cost_of_Capital_Data.xlsx
+++ b/Walmart_Cost_of_Capital_Data.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="114">
   <si>
     <t xml:space="preserve">Estimating Walmart's cost of capital: summary of results</t>
   </si>
@@ -106,21 +106,6 @@
   </si>
   <si>
     <t xml:space="preserve">Q7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Color key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue text: input taken from the Walmart case study</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Black text: formula calculated on the same sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Green text: value linked from another sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yellow fill: key result</t>
   </si>
   <si>
     <t xml:space="preserve">Question 2: Walmart sources of financing</t>
@@ -397,7 +382,7 @@
     <numFmt numFmtId="169" formatCode="0.00"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -422,16 +407,13 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF1F3864"/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
       <sz val="10"/>
-      <color rgb="FF595959"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -439,104 +421,17 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF008000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF008000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF595959"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF333333"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -550,19 +445,15 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom/>
+      <top/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top style="thin">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="double"/>
+      <top style="thin"/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -591,7 +482,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -604,23 +495,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -628,111 +515,51 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -740,23 +567,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -769,66 +584,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFF2F2F2"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD9E1F2"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF595959"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF1F3864"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -1012,7 +767,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1021,7 +776,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1046,178 +801,153 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="5" t="n">
         <f aca="false">'Q2 Financing Sources'!B18</f>
         <v>139661</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="5" t="n">
         <f aca="false">'Q2 Financing Sources'!B26</f>
         <v>79634</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="5" t="n">
         <f aca="false">'Q2 Financing Sources'!B28</f>
         <v>219295</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8" t="n">
         <f aca="false">'Q3 Cost of Debt'!B10</f>
         <v>0.0353</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="9" t="n">
         <f aca="false">'Q4 Cost of Equity'!B12</f>
         <v>0.106091</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <f aca="false">'Q5 Capital Structure'!D5</f>
         <v>0.636863585581067</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="8" t="n">
         <f aca="false">'Q5 Capital Structure'!D6</f>
         <v>0.363136414418933</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">'Q5 Capital Structure'!B10</f>
         <v>1.75378607127609</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="12" t="n">
         <f aca="false">'Q6-Q7 WACC &amp; MARR'!B15</f>
         <v>0.0549368430789576</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="13" t="n">
+      <c r="B14" s="12" t="n">
         <f aca="false">'Q6-Q7 WACC &amp; MARR'!B17</f>
         <v>0.0549368430789576</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1244,290 +974,281 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="19" t="n">
+      <c r="B6" s="5" t="n">
         <v>47060</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="8" t="n">
         <f aca="false">B6/$B$28</f>
         <v>0.214596776032285</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="19" t="n">
+      <c r="A7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="5" t="n">
         <v>5225</v>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="8" t="n">
         <f aca="false">B7/$B$28</f>
         <v>0.0238263526300189</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="19" t="n">
+      <c r="A8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="5" t="n">
         <v>22159</v>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="8" t="n">
         <f aca="false">B8/$B$28</f>
         <v>0.101046535488725</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="19" t="n">
+      <c r="A9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="5" t="n">
         <v>2605</v>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="8" t="n">
         <f aca="false">B9/$B$28</f>
         <v>0.011878975808842</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="19" t="n">
+      <c r="A10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="5" t="n">
         <v>428</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="8" t="n">
         <f aca="false">B10/$B$28</f>
         <v>0.0019517088852915</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="22" t="n">
+      <c r="A11" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="14" t="n">
         <f aca="false">SUM(B6:B10)</f>
         <v>77477</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="15" t="n">
         <f aca="false">B11/$B$28</f>
         <v>0.353300348845163</v>
       </c>
-      <c r="D11" s="24"/>
+      <c r="D11" s="13"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
+      <c r="A13" s="11" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="19" t="n">
+      <c r="A14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="5" t="n">
         <v>50203</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="8" t="n">
         <f aca="false">B14/$B$28</f>
         <v>0.228929068150209</v>
       </c>
-      <c r="D14" s="8" t="s">
-        <v>47</v>
+      <c r="D14" s="7" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" s="19" t="n">
+      <c r="A15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="5" t="n">
         <v>11981</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="8" t="n">
         <f aca="false">B15/$B$28</f>
         <v>0.0546341685856951</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" s="22" t="n">
+      <c r="A16" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="14" t="n">
         <f aca="false">SUM(B14:B15)</f>
         <v>62184</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="15" t="n">
         <f aca="false">B16/$B$28</f>
         <v>0.283563236735904</v>
       </c>
-      <c r="D16" s="24"/>
+      <c r="D16" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18" s="22" t="n">
+      <c r="A18" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="14" t="n">
         <f aca="false">B11+B16</f>
         <v>139661</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="15" t="n">
         <f aca="false">B18/$B$28</f>
         <v>0.636863585581067</v>
       </c>
-      <c r="D18" s="25" t="s">
-        <v>51</v>
+      <c r="D18" s="16" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
+      <c r="A20" s="11" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="19" t="n">
+      <c r="A21" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="5" t="n">
         <v>3253</v>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="8" t="n">
         <f aca="false">B21/$B$28</f>
         <v>0.0148338995417132</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="19" t="n">
+      <c r="A22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="5" t="n">
         <v>80785</v>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="8" t="n">
         <f aca="false">B22/$B$28</f>
         <v>0.368385052098771</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="19" t="n">
+      <c r="A23" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="5" t="n">
         <v>-11542</v>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="8" t="n">
         <f aca="false">B23/$B$28</f>
         <v>-0.0526322989580246</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="B24" s="22" t="n">
+      <c r="A24" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="14" t="n">
         <f aca="false">SUM(B21:B23)</f>
         <v>72496</v>
       </c>
-      <c r="C24" s="23" t="n">
+      <c r="C24" s="15" t="n">
         <f aca="false">B24/$B$28</f>
         <v>0.33058665268246</v>
       </c>
-      <c r="D24" s="24"/>
+      <c r="D24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B25" s="19" t="n">
+      <c r="A25" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="5" t="n">
         <v>7138</v>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="8" t="n">
         <f aca="false">B25/$B$28</f>
         <v>0.0325497617364737</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26" s="22" t="n">
+      <c r="A26" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="14" t="n">
         <f aca="false">B24+B25</f>
         <v>79634</v>
       </c>
-      <c r="C26" s="23" t="n">
+      <c r="C26" s="15" t="n">
         <f aca="false">B26/$B$28</f>
         <v>0.363136414418933</v>
       </c>
-      <c r="D26" s="25" t="s">
-        <v>59</v>
+      <c r="D26" s="16" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="B28" s="27" t="n">
+      <c r="A28" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="14" t="n">
         <f aca="false">B18+B26</f>
         <v>219295</v>
       </c>
-      <c r="C28" s="28" t="n">
+      <c r="C28" s="15" t="n">
         <f aca="false">B28/$B$28</f>
         <v>1</v>
       </c>
-      <c r="D28" s="29"/>
+      <c r="D28" s="13"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B30" s="19" t="n">
+      <c r="A30" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="5" t="n">
         <v>219295</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="30" t="n">
+      <c r="A31" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="5" t="n">
         <f aca="false">B28-B30</f>
         <v>0</v>
       </c>
@@ -1558,89 +1279,89 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="6" t="n">
+      <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="5" t="n">
         <f aca="false">'Q2 Financing Sources'!B14</f>
         <v>50203</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="8" t="n">
         <f aca="false">B5/$B$7</f>
         <v>0.807329859771002</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>69</v>
+      <c r="D5" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B6" s="6" t="n">
+      <c r="A6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="5" t="n">
         <f aca="false">'Q2 Financing Sources'!B15</f>
         <v>11981</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="8" t="n">
         <f aca="false">B6/$B$7</f>
         <v>0.192670140228998</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>71</v>
+      <c r="D6" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="22" t="n">
+      <c r="A7" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="14" t="n">
         <f aca="false">SUM(B5:B6)</f>
         <v>62184</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="15" t="n">
         <f aca="false">B7/$B$7</f>
         <v>1</v>
       </c>
-      <c r="D7" s="31"/>
-      <c r="E7" s="24"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>3</v>
@@ -1648,18 +1369,18 @@
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B10" s="32" t="n">
+      <c r="A10" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B10" s="12" t="n">
         <v>0.0353</v>
       </c>
-      <c r="E10" s="8" t="s">
-        <v>75</v>
+      <c r="E10" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1686,112 +1407,112 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B5" s="33" t="n">
+      <c r="A5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="18" t="n">
         <v>0.71</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="8" t="n">
         <v>0.0265</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>75</v>
+      <c r="C6" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="34" t="n">
+      <c r="A7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="8" t="n">
         <v>0.1349</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>75</v>
+      <c r="C7" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B8" s="34" t="n">
+      <c r="A8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <v>0.0228</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>75</v>
+      <c r="C8" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="20" t="n">
+      <c r="A11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="8" t="n">
         <f aca="false">B7-B8</f>
         <v>0.1121</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>86</v>
+      <c r="C11" s="7" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B12" s="35" t="n">
+      <c r="A12" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="19" t="n">
         <f aca="false">B6+B5*B11</f>
         <v>0.106091</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>88</v>
+      <c r="C12" s="7" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
+      <c r="A14" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1821,107 +1542,107 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B5" s="6" t="n">
+      <c r="A5" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="5" t="n">
         <f aca="false">'Q2 Financing Sources'!B18</f>
         <v>139661</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <f aca="false">'Q3 Cost of Debt'!B10</f>
         <v>0.0353</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="8" t="n">
         <f aca="false">B5/$B$7</f>
         <v>0.636863585581067</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="6" t="n">
+      <c r="A6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="5" t="n">
         <f aca="false">'Q2 Financing Sources'!B26</f>
         <v>79634</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="9" t="n">
         <f aca="false">'Q4 Cost of Equity'!B12</f>
         <v>0.106091</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="8" t="n">
         <f aca="false">B6/$B$7</f>
         <v>0.363136414418933</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
-        <v>97</v>
-      </c>
-      <c r="B7" s="27" t="n">
+      <c r="A7" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="14" t="n">
         <f aca="false">B5+B6</f>
         <v>219295</v>
       </c>
-      <c r="C7" s="29"/>
-      <c r="D7" s="28" t="n">
+      <c r="C7" s="13"/>
+      <c r="D7" s="15" t="n">
         <f aca="false">D5+D6</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="37" t="n">
+      <c r="B10" s="21" t="n">
         <f aca="false">B5/B6</f>
         <v>1.75378607127609</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>99</v>
+      <c r="C10" s="7" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B11" s="38" t="n">
+      <c r="A11" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="22" t="n">
         <f aca="false">B10</f>
         <v>1.75378607127609</v>
       </c>
@@ -1950,155 +1671,155 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B5" s="9" t="n">
+      <c r="A5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="8" t="n">
         <f aca="false">'Q5 Capital Structure'!D6</f>
         <v>0.363136414418933</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>104</v>
+      <c r="C5" s="7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B6" s="10" t="n">
+      <c r="A6" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="9" t="n">
         <f aca="false">'Q4 Cost of Equity'!B12</f>
         <v>0.106091</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>105</v>
+      <c r="C6" s="7" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B7" s="9" t="n">
+      <c r="A7" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="8" t="n">
         <f aca="false">'Q5 Capital Structure'!D5</f>
         <v>0.636863585581067</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>104</v>
+      <c r="C7" s="7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="9" t="n">
+      <c r="A8" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <f aca="false">'Q3 Cost of Debt'!B10</f>
         <v>0.0353</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>108</v>
+      <c r="C8" s="7" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B9" s="34" t="n">
+      <c r="A9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="8" t="n">
         <v>0.27</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>75</v>
+      <c r="C9" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>3</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B12" s="20" t="n">
+      <c r="A12" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="8" t="n">
         <f aca="false">B8*(1-B9)</f>
         <v>0.025769</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>111</v>
+      <c r="C12" s="7" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="B13" s="20" t="n">
+      <c r="A13" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="8" t="n">
         <f aca="false">B5*B6</f>
         <v>0.0385255053421191</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>113</v>
+      <c r="C13" s="7" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B14" s="20" t="n">
+      <c r="A14" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="8" t="n">
         <f aca="false">B7*B12</f>
         <v>0.0164113377368385</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>115</v>
+      <c r="C14" s="7" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="B15" s="39" t="n">
+      <c r="A15" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B15" s="15" t="n">
         <f aca="false">B13+B14</f>
         <v>0.0549368430789576</v>
       </c>
-      <c r="C15" s="40" t="s">
-        <v>117</v>
+      <c r="C15" s="16" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="41" t="n">
+      <c r="B17" s="12" t="n">
         <f aca="false">B15</f>
         <v>0.0549368430789576</v>
       </c>
-      <c r="C17" s="8" t="s">
-        <v>118</v>
+      <c r="C17" s="7" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>